<commit_message>
scripting as been completed which include handover file processing and also hide the credentials
</commit_message>
<xml_diff>
--- a/cleaned_handover/SBSA/Panel L/Handover_APT_LSW/Mar 2026/Standard_Bank_Panel_L_Handover_20260319.xlsx
+++ b/cleaned_handover/SBSA/Panel L/Handover_APT_LSW/Mar 2026/Standard_Bank_Panel_L_Handover_20260319.xlsx
@@ -442,7 +442,7 @@
     <t xml:space="preserve">Prescription Date</t>
   </si>
   <si>
-    <t xml:space="preserve">10057675692</t>
+    <t xml:space="preserve">10050000602</t>
   </si>
   <si>
     <t xml:space="preserve">STA614</t>
@@ -808,10 +808,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.93"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="24.03"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="20.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="13.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="34" style="1" width="11.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="58" min="58" style="1" width="12.1"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="78" min="78" style="1" width="36.33"/>

</xml_diff>